<commit_message>
graduell wärmer in Buch 4 ab 4-3-xx
</commit_message>
<xml_diff>
--- a/Stats.xlsx
+++ b/Stats.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jakof-my.sharepoint.com/personal/andreas_jakof_eu/Documents/UntilTheEnd/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="57" documentId="8_{4435BF9B-1680-49F8-AF21-CC181DBFEE0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{801C9DE0-52BA-4468-8066-F43D97EC189A}"/>
+  <xr:revisionPtr revIDLastSave="59" documentId="8_{4435BF9B-1680-49F8-AF21-CC181DBFEE0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C3950EEF-4DCD-4048-8A20-34BA445DCCF9}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{A3D688E1-50A5-4922-B0AE-A46EBCE519BE}"/>
+    <workbookView minimized="1" xWindow="3900" yWindow="3900" windowWidth="28800" windowHeight="15345" xr2:uid="{A3D688E1-50A5-4922-B0AE-A46EBCE519BE}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -213,7 +213,7 @@
                   <c:v>46085.472222222219</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>46088</c:v>
+                  <c:v>46088.720833333333</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -231,7 +231,7 @@
                   <c:v>17447</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>18805</c:v>
+                  <c:v>19772</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -502,7 +502,7 @@
                   <c:v>46085.472222222219</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>46088</c:v>
+                  <c:v>46088.720833333333</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -791,7 +791,7 @@
                   <c:v>46085.472222222219</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>46088</c:v>
+                  <c:v>46088.720833333333</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1932,7 +1932,7 @@
                   <c:v>46085.472222222219</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>46088</c:v>
+                  <c:v>46088.720833333333</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -6686,10 +6686,10 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
-        <v>46088</v>
+        <v>46088.720833333333</v>
       </c>
       <c r="B4" s="2">
-        <v>18805</v>
+        <v>19772</v>
       </c>
       <c r="C4">
         <v>90</v>

</xml_diff>